<commit_message>
Fixed bug regarding allocation
</commit_message>
<xml_diff>
--- a/participants.xlsx
+++ b/participants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Svelte Learning\hostel-allotment-system\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\hostel-allotment-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F4026D5-4713-4E30-A614-118B254DB5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1F3CA85-9268-4CA4-8742-ED5B9C29A207}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="19386" windowHeight="12186" xr2:uid="{AE71973D-1FCC-4A06-ABEC-75039B5E8AFF}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="12">
   <si>
     <t>Participant Name</t>
   </si>
@@ -443,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DD546A4-1A36-48F9-BF03-F84036283ECE}">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <cols>
     <col min="1" max="1" width="16.3515625" customWidth="1"/>
@@ -521,6 +521,70 @@
         <v>6</v>
       </c>
     </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A10" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A12" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A13" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A14" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.5">
+      <c r="A17" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" t="s">
+        <v>6</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>